<commit_message>
Prueba de calidad de Vinos
</commit_message>
<xml_diff>
--- a/data/resultado.xlsx
+++ b/data/resultado.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,13 +452,13 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>5.2</v>
+        <v>6.5</v>
       </c>
       <c r="B2" t="n">
-        <v>10.5</v>
+        <v>11.2</v>
       </c>
       <c r="C2" t="n">
-        <v>1.3</v>
+        <v>3.1</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -466,13 +466,13 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>6.8</v>
+        <v>7.1</v>
       </c>
       <c r="B3" t="n">
-        <v>12.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -480,15 +480,57 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3.1</v>
+        <v>5.9</v>
       </c>
       <c r="B4" t="n">
-        <v>8.9</v>
+        <v>12</v>
       </c>
       <c r="C4" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="D4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B5" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="B6" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="B7" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="C7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D7" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>